<commit_message>
Rebuild the cumulative row from daily measurements instead of a carry file
The 7/18-onward cumulative was kept in cum.json and each run added
yesterday to it. Regenerating the report three times this morning added
7/26 three times, reporting 16,290,866 yen of cumulative sales against an
actual 13,041,944. Every other row recomputes from scratch, so only the
cumulative was affected.

The cumulative now sums the measured dailies on every run and asserts that
the total matches the sum of its component days, so running twice produces
the same number. Whole-store ad spend also moves from summing campaigns to
Meta's account-level daily totals, which cannot silently drop a campaign.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JNTxDUfjQsrckfss7YKHj
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-27.xlsx
+++ b/data/reports/report-2026-07-27.xlsx
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -696,17 +696,17 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>626620</v>
+        <v>626704</v>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="5" t="n">
-        <v>576470</v>
+        <v>576498</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>559921</v>
+        <v>559933</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>471127</v>
+        <v>471129</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
@@ -721,17 +721,17 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>518466</v>
+        <v>518382</v>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="5" t="n">
-        <v>435424</v>
+        <v>435396</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>478218</v>
+        <v>478206</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>452210</v>
+        <v>452207</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
@@ -779,17 +779,17 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>461772</v>
+        <v>461688</v>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="5" t="n">
-        <v>385129</v>
+        <v>385101</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>426246</v>
+        <v>426234</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>406759</v>
+        <v>406756</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
@@ -864,22 +864,22 @@
         <v>479375</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>626620</v>
+        <v>626704</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>518466</v>
+        <v>518382</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>0.3192</v>
+        <v>0.3191</v>
       </c>
       <c r="G14" s="6" t="n">
         <v>56694</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>461772</v>
+        <v>461688</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>0.2843</v>
+        <v>0.2842</v>
       </c>
     </row>
     <row r="15">
@@ -895,10 +895,10 @@
         <v>1287738</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>1729409</v>
+        <v>1729493</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>1306273</v>
+        <v>1306189</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>0.3021</v>
@@ -907,7 +907,7 @@
         <v>150887</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>1155386</v>
+        <v>1155302</v>
       </c>
       <c r="I15" s="7" t="n">
         <v>0.2672</v>
@@ -926,10 +926,10 @@
         <v>3157189</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>3919446</v>
+        <v>3919530</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>3347527</v>
+        <v>3347443</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>0.3211</v>
@@ -938,7 +938,7 @@
         <v>363803</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>2983724</v>
+        <v>2983640</v>
       </c>
       <c r="I16" s="7" t="n">
         <v>0.2862</v>
@@ -957,10 +957,10 @@
         <v>11369539</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>14133800</v>
+        <v>14133884</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>13566306</v>
+        <v>13566222</v>
       </c>
       <c r="F17" s="7" t="n">
         <v>0.3472</v>
@@ -969,7 +969,7 @@
         <v>1363531</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>12202775</v>
+        <v>12202691</v>
       </c>
       <c r="I17" s="7" t="n">
         <v>0.3123</v>
@@ -982,28 +982,28 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>16290866</v>
+        <v>13041944</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>4887073</v>
+        <v>3916512</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>6201349</v>
+        <v>4948380</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>5202444</v>
+        <v>4177052</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>0.3193</v>
+        <v>0.3203</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>568551</v>
+        <v>455164</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>4633893</v>
+        <v>3721888</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>0.2844</v>
+        <v>0.2854</v>
       </c>
     </row>
     <row r="20">
@@ -1080,6 +1080,27 @@
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>・★増額候補（自分の目標MER超え × 消化率95%以上）: 4WAY 取り付けOK (3.73&gt;3.30・103%)・害虫ブロッカー(2.91&gt;2.31・100%)・形状記憶日傘(3.44&gt;2.58・98%)・ナノガラス脱毛パッド(2.51&gt;2.17・100%)・卓上冷感クーラー(3.73&gt;3.16・98%)・5WAY腰掛けファン(4.59&gt;3.59・102%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>・⚠️訂正: 7/27朝に一度お渡ししたファイルの「7/18〜累積」行が誤っていました（売上16,290,866円等）。累積を繰り越しファイルへの加算方式で作っていたため、生成スクリプトを3回走らせた分だけ7/26が3重計上されていました。本ファイルは累積を日次実測から毎回積み直す方式に変更し、日次合計との一致を自動チェックしています（他の行は元から毎回再計算のため影響なし）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>・★全店の広告費をキャンペーン合算からMetaのアカウントレベル日次実測に変更（取りこぼしが構造的に起きない）。差は7日で84円</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>・★7/18〜累積の原価は全日を現行（7/25改定後）の原価表で評価している。前回ファイルの8日累積3,448,948円との差−11,811円は、この基準統一とディスペンサーのバリエーション別原価の修正による</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3195,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>ナノバブルシャワーヘッド</t>
+          <t>ネックマッサージャー</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
@@ -3219,7 +3240,7 @@
       </c>
       <c r="R24" s="4" t="inlineStr"/>
       <c r="S24" s="6" t="n">
-        <v>51975</v>
+        <v>6946</v>
       </c>
       <c r="T24" s="4" t="inlineStr"/>
       <c r="U24" s="4" t="inlineStr"/>
@@ -3245,7 +3266,7 @@
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>リカバリーサンダル</t>
+          <t>姿勢サポートベルト</t>
         </is>
       </c>
       <c r="B25" s="16" t="n">
@@ -3290,7 +3311,7 @@
       </c>
       <c r="R25" s="15" t="inlineStr"/>
       <c r="S25" s="16" t="n">
-        <v>18697</v>
+        <v>4551</v>
       </c>
       <c r="T25" s="15" t="inlineStr"/>
       <c r="U25" s="15" t="inlineStr"/>
@@ -3316,7 +3337,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>ネックマッサージャー</t>
+          <t>ナノバブルシャワーヘッド</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
@@ -3361,7 +3382,7 @@
       </c>
       <c r="R26" s="4" t="inlineStr"/>
       <c r="S26" s="6" t="n">
-        <v>6946</v>
+        <v>51975</v>
       </c>
       <c r="T26" s="4" t="inlineStr"/>
       <c r="U26" s="4" t="inlineStr"/>
@@ -3387,7 +3408,7 @@
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>姿勢サポートベルト</t>
+          <t>リカバリーサンダル</t>
         </is>
       </c>
       <c r="B27" s="16" t="n">
@@ -3432,7 +3453,7 @@
       </c>
       <c r="R27" s="15" t="inlineStr"/>
       <c r="S27" s="16" t="n">
-        <v>4551</v>
+        <v>18697</v>
       </c>
       <c r="T27" s="15" t="inlineStr"/>
       <c r="U27" s="15" t="inlineStr"/>

</xml_diff>